<commit_message>
Add: pieces and board reading from excel
</commit_message>
<xml_diff>
--- a/itdm/data.xlsx
+++ b/itdm/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\adrian\itdc\70160513-Introduction-to-decision-making\itdm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9E19905-282A-4528-8275-25696D157216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA1D12DF-543F-4713-A39B-43FA37E005F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{D04539F6-9DBE-4AA4-A75F-D46447C73DF5}"/>
+    <workbookView xWindow="1125" yWindow="1125" windowWidth="11040" windowHeight="11775" activeTab="1" xr2:uid="{D04539F6-9DBE-4AA4-A75F-D46447C73DF5}"/>
   </bookViews>
   <sheets>
     <sheet name="Pieces" sheetId="1" r:id="rId1"/>
@@ -426,11 +426,11 @@
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1">
-        <v>2</v>
+        <v>200</v>
       </c>
       <c r="C1" s="1">
         <f>$A1</f>
-        <v>2</v>
+        <v>200</v>
       </c>
       <c r="H1" s="1">
         <f>$A2</f>
@@ -992,68 +992,77 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD0C2727-F031-4F02-AB0E-CAE8E0EBF1D0}">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B1">
-        <v>2</v>
-      </c>
-      <c r="C1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
       <c r="G2">
         <v>1</v>
       </c>
-      <c r="H2">
-        <v>1</v>
-      </c>
-      <c r="I2">
-        <v>1</v>
-      </c>
-      <c r="J2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>6</v>
-      </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="J4">
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="E8">
         <v>1</v>
       </c>
     </row>

</xml_diff>